<commit_message>
Updated with better layout for Figure, but README not re-run
</commit_message>
<xml_diff>
--- a/_readme/datafiles.xlsx
+++ b/_readme/datafiles.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="335" uniqueCount="103">
   <si>
     <t xml:space="preserve">Filename</t>
   </si>
@@ -323,6 +323,12 @@
   </si>
   <si>
     <t xml:space="preserve">./data/stata-licenses-by-country.xlsx</t>
+  </si>
+  <si>
+    <t xml:space="preserve">./data/table.aea.software_by_year.csv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vilhuber (2020a)</t>
   </si>
 </sst>
 </file>
@@ -611,7 +617,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E83"/>
+  <dimension ref="A1:E84"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="54.68"/>
@@ -765,7 +771,7 @@
       <c r="D9" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="0" t="n">
+      <c r="E9" s="1" t="n">
         <v>24</v>
       </c>
     </row>
@@ -1901,10 +1907,10 @@
       <c r="C76" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="D76" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="E76" s="0" t="n">
+      <c r="D76" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E76" s="1" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1952,7 +1958,7 @@
       <c r="D79" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E79" s="0" t="n">
+      <c r="E79" s="1" t="n">
         <v>22</v>
       </c>
     </row>
@@ -1969,7 +1975,7 @@
       <c r="D80" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="E80" s="0" t="n">
+      <c r="E80" s="1" t="n">
         <v>23</v>
       </c>
     </row>
@@ -2013,6 +2019,23 @@
       </c>
       <c r="D83" s="1" t="s">
         <v>8</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A84" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="D84" s="0" t="s">
+        <v>8</v>
+      </c>
+      <c r="E84" s="0" t="n">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>